<commit_message>
Added Test Case scenario Library Management System
</commit_message>
<xml_diff>
--- a/LMS TestCases.xlsx
+++ b/LMS TestCases.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Saurabh Mishra\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3AC541E-9A81-4D15-8A41-885BF36AF581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30B2435-A9D1-4B29-A533-8EF3486024E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{313A250A-E99B-40BD-A3F8-AE5FBCBF32A4}"/>
   </bookViews>
   <sheets>
     <sheet name="ADD USER" sheetId="1" r:id="rId1"/>
     <sheet name="UPDATE USER" sheetId="2" r:id="rId2"/>
-    <sheet name="UPDATE USER NEW" sheetId="3" r:id="rId3"/>
+    <sheet name="USER LOGIN" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1039" uniqueCount="593">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1039" uniqueCount="596">
   <si>
     <t>APPLICATION NAME</t>
   </si>
@@ -1815,6 +1815,15 @@
   </si>
   <si>
     <t>Mishra@</t>
+  </si>
+  <si>
+    <t>USER LOGIN</t>
+  </si>
+  <si>
+    <t>2.1 MEMBER LOGIN</t>
+  </si>
+  <si>
+    <t>USER SHOULD BE REGISTERED AND NAVIGATED TO LOGIN PAGE</t>
   </si>
 </sst>
 </file>
@@ -5081,7 +5090,7 @@
         <v>23</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>11</v>
+        <v>593</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -5089,7 +5098,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>192</v>
+        <v>594</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5097,7 +5106,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>193</v>
+        <v>595</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>